<commit_message>
Analyse des données 2012
</commit_message>
<xml_diff>
--- a/server/template/Horaires.xlsx
+++ b/server/template/Horaires.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30610"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A84856CB-FAD3-41C1-BE40-F23D4AA911B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{64357C21-089C-4E18-ACFB-11D797621368}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="447" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="448" uniqueCount="30">
   <si>
     <t>Janvier</t>
   </si>
@@ -122,6 +122,9 @@
   <si>
     <t>Total</t>
   </si>
+  <si>
+    <t>Du</t>
+  </si>
 </sst>
 </file>
 
@@ -200,7 +203,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="26">
+  <borders count="22">
     <border>
       <left/>
       <right/>
@@ -428,63 +431,6 @@
       <left style="thin">
         <color rgb="FF000000"/>
       </left>
-      <right style="medium">
-        <color rgb="FF000000"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
       <right/>
       <top/>
       <bottom/>
@@ -529,11 +475,26 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="71">
+  <cellXfs count="67">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -643,16 +604,10 @@
     <xf numFmtId="0" fontId="1" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -661,10 +616,10 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -679,71 +634,65 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" textRotation="180" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="180" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="180" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" textRotation="180" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="180" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="180" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1098,7 +1047,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:39" ht="61.5" customHeight="1">
-      <c r="A1" s="64" t="s">
+      <c r="A1" s="54" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1">
@@ -1195,16 +1144,16 @@
         <v>31</v>
       </c>
       <c r="AG1" s="5"/>
-      <c r="AH1" s="60" t="s">
+      <c r="AH1" s="50" t="s">
         <v>0</v>
       </c>
-      <c r="AI1" s="61"/>
+      <c r="AI1" s="51"/>
       <c r="AK1" s="6" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="2" spans="1:39" ht="61.5" customHeight="1">
-      <c r="A2" s="65"/>
+      <c r="A2" s="55"/>
       <c r="B2" s="7" t="s">
         <v>2</v>
       </c>
@@ -1299,12 +1248,12 @@
         <v>4</v>
       </c>
       <c r="AG2" s="5"/>
-      <c r="AH2" s="62"/>
-      <c r="AI2" s="63"/>
-      <c r="AK2" s="53" t="s">
+      <c r="AH2" s="52"/>
+      <c r="AI2" s="53"/>
+      <c r="AK2" s="56" t="s">
         <v>9</v>
       </c>
-      <c r="AL2" s="54"/>
+      <c r="AL2" s="57"/>
     </row>
     <row r="3" spans="1:39" ht="61.5" customHeight="1">
       <c r="A3" s="12" t="s">
@@ -1381,10 +1330,10 @@
         <f>SUM(B3:AF3)</f>
         <v>148</v>
       </c>
-      <c r="AK3" s="55" t="s">
+      <c r="AK3" s="58" t="s">
         <v>11</v>
       </c>
-      <c r="AL3" s="56"/>
+      <c r="AL3" s="59"/>
     </row>
     <row r="4" spans="1:39" ht="61.5" customHeight="1">
       <c r="A4" s="17" t="s">
@@ -1429,10 +1378,10 @@
         <f t="shared" ref="AI4" si="0">SUM(B4:AF4)</f>
         <v>0</v>
       </c>
-      <c r="AK4" s="57" t="s">
+      <c r="AK4" s="60" t="s">
         <v>13</v>
       </c>
-      <c r="AL4" s="58"/>
+      <c r="AL4" s="61"/>
     </row>
     <row r="5" spans="1:39" ht="61.5" customHeight="1">
       <c r="B5" s="25"/>
@@ -1467,13 +1416,13 @@
       <c r="AE5" s="25"/>
       <c r="AF5" s="25"/>
       <c r="AG5" s="5"/>
-      <c r="AK5" s="59" t="s">
+      <c r="AK5" s="62" t="s">
         <v>14</v>
       </c>
-      <c r="AL5" s="59"/>
+      <c r="AL5" s="62"/>
     </row>
     <row r="6" spans="1:39" ht="61.5" customHeight="1">
-      <c r="A6" s="64" t="s">
+      <c r="A6" s="54" t="s">
         <v>15</v>
       </c>
       <c r="B6" s="2">
@@ -1564,15 +1513,15 @@
       <c r="AE6" s="25"/>
       <c r="AF6" s="25"/>
       <c r="AG6" s="5"/>
-      <c r="AH6" s="60" t="s">
+      <c r="AH6" s="50" t="s">
         <v>15</v>
       </c>
-      <c r="AI6" s="61"/>
-      <c r="AK6" s="59"/>
-      <c r="AL6" s="59"/>
+      <c r="AI6" s="51"/>
+      <c r="AK6" s="62"/>
+      <c r="AL6" s="62"/>
     </row>
     <row r="7" spans="1:39" ht="61.5" customHeight="1">
-      <c r="A7" s="65"/>
+      <c r="A7" s="55"/>
       <c r="B7" s="8" t="s">
         <v>5</v>
       </c>
@@ -1661,10 +1610,10 @@
       <c r="AE7" s="25"/>
       <c r="AF7" s="25"/>
       <c r="AG7" s="5"/>
-      <c r="AH7" s="62"/>
-      <c r="AI7" s="63"/>
-      <c r="AK7" s="66"/>
-      <c r="AL7" s="66"/>
+      <c r="AH7" s="52"/>
+      <c r="AI7" s="53"/>
+      <c r="AK7" s="47"/>
+      <c r="AL7" s="47"/>
     </row>
     <row r="8" spans="1:39" ht="61.5" customHeight="1">
       <c r="A8" s="12" t="s">
@@ -1824,10 +1773,10 @@
       <c r="AE10" s="25"/>
       <c r="AF10" s="25"/>
       <c r="AG10" s="5"/>
-      <c r="AK10" s="67"/>
+      <c r="AK10" s="48"/>
     </row>
     <row r="11" spans="1:39" ht="61.5" customHeight="1">
-      <c r="A11" s="64" t="s">
+      <c r="A11" s="54" t="s">
         <v>16</v>
       </c>
       <c r="B11" s="2">
@@ -1914,7 +1863,7 @@
       <c r="AC11" s="3">
         <v>28</v>
       </c>
-      <c r="AD11" s="39">
+      <c r="AD11" s="37">
         <v>29</v>
       </c>
       <c r="AE11" s="2">
@@ -1924,15 +1873,15 @@
         <v>31</v>
       </c>
       <c r="AG11" s="5"/>
-      <c r="AH11" s="60" t="s">
+      <c r="AH11" s="50" t="s">
         <v>16</v>
       </c>
-      <c r="AI11" s="61"/>
-      <c r="AK11" s="68"/>
-      <c r="AL11" s="68"/>
+      <c r="AI11" s="51"/>
+      <c r="AK11" s="49"/>
+      <c r="AL11" s="49"/>
     </row>
     <row r="12" spans="1:39" ht="61.5" customHeight="1">
-      <c r="A12" s="65"/>
+      <c r="A12" s="55"/>
       <c r="B12" s="8" t="s">
         <v>5</v>
       </c>
@@ -2017,7 +1966,7 @@
       <c r="AC12" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="AD12" s="40" t="s">
+      <c r="AD12" s="38" t="s">
         <v>5</v>
       </c>
       <c r="AE12" s="8" t="s">
@@ -2027,10 +1976,10 @@
         <v>7</v>
       </c>
       <c r="AG12" s="5"/>
-      <c r="AH12" s="62"/>
-      <c r="AI12" s="63"/>
-      <c r="AK12" s="68"/>
-      <c r="AL12" s="68"/>
+      <c r="AH12" s="52"/>
+      <c r="AI12" s="53"/>
+      <c r="AK12" s="49"/>
+      <c r="AL12" s="49"/>
     </row>
     <row r="13" spans="1:39" ht="61.5" customHeight="1">
       <c r="A13" s="12" t="s">
@@ -2096,7 +2045,7 @@
       </c>
       <c r="AB13" s="10"/>
       <c r="AC13" s="10"/>
-      <c r="AD13" s="43"/>
+      <c r="AD13" s="41"/>
       <c r="AE13" s="8">
         <v>9.25</v>
       </c>
@@ -2109,8 +2058,8 @@
         <f>SUM(B13:AF13)</f>
         <v>157.25</v>
       </c>
-      <c r="AK13" s="68"/>
-      <c r="AL13" s="68"/>
+      <c r="AK13" s="49"/>
+      <c r="AL13" s="49"/>
     </row>
     <row r="14" spans="1:39" ht="61.5" customHeight="1">
       <c r="A14" s="17" t="s">
@@ -2144,7 +2093,7 @@
       <c r="AA14" s="19"/>
       <c r="AB14" s="20"/>
       <c r="AC14" s="20"/>
-      <c r="AD14" s="44"/>
+      <c r="AD14" s="42"/>
       <c r="AE14" s="19"/>
       <c r="AF14" s="36"/>
       <c r="AG14" s="5"/>
@@ -2155,8 +2104,8 @@
         <f t="shared" ref="AI14" si="2">SUM(B14:AF14)</f>
         <v>0</v>
       </c>
-      <c r="AK14" s="68"/>
-      <c r="AL14" s="68"/>
+      <c r="AK14" s="49"/>
+      <c r="AL14" s="49"/>
     </row>
     <row r="15" spans="1:39" ht="61.5" customHeight="1">
       <c r="B15" s="25"/>
@@ -2191,11 +2140,11 @@
       <c r="AE15" s="25"/>
       <c r="AF15" s="25"/>
       <c r="AG15" s="5"/>
-      <c r="AK15" s="68"/>
-      <c r="AL15" s="68"/>
+      <c r="AK15" s="49"/>
+      <c r="AL15" s="49"/>
     </row>
     <row r="16" spans="1:39" ht="61.5" customHeight="1">
-      <c r="A16" s="64" t="s">
+      <c r="A16" s="54" t="s">
         <v>17</v>
       </c>
       <c r="B16" s="2">
@@ -2290,19 +2239,19 @@
       </c>
       <c r="AF16" s="25"/>
       <c r="AG16" s="5"/>
-      <c r="AH16" s="60" t="s">
+      <c r="AH16" s="50" t="s">
         <v>17</v>
       </c>
-      <c r="AI16" s="61"/>
-      <c r="AK16" s="69" t="s">
+      <c r="AI16" s="51"/>
+      <c r="AK16" s="64" t="s">
         <v>18</v>
       </c>
-      <c r="AL16" s="70" t="s">
+      <c r="AL16" s="63" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="17" spans="1:42" ht="61.5" customHeight="1">
-      <c r="A17" s="65"/>
+      <c r="A17" s="55"/>
       <c r="B17" s="8" t="s">
         <v>8</v>
       </c>
@@ -2390,15 +2339,15 @@
       <c r="AD17" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="AE17" s="42" t="s">
+      <c r="AE17" s="40" t="s">
         <v>2</v>
       </c>
       <c r="AF17" s="25"/>
       <c r="AG17" s="5"/>
-      <c r="AH17" s="62"/>
-      <c r="AI17" s="63"/>
-      <c r="AK17" s="69"/>
-      <c r="AL17" s="70"/>
+      <c r="AH17" s="52"/>
+      <c r="AI17" s="53"/>
+      <c r="AK17" s="64"/>
+      <c r="AL17" s="63"/>
     </row>
     <row r="18" spans="1:42" ht="61.5" customHeight="1">
       <c r="A18" s="12" t="s">
@@ -2461,7 +2410,7 @@
       <c r="AD18" s="8">
         <v>9.25</v>
       </c>
-      <c r="AE18" s="41">
+      <c r="AE18" s="39">
         <v>9.25</v>
       </c>
       <c r="AF18" s="25"/>
@@ -2473,8 +2422,8 @@
         <f>SUM(B18:AF18)</f>
         <v>131.25</v>
       </c>
-      <c r="AK18" s="69"/>
-      <c r="AL18" s="70"/>
+      <c r="AK18" s="64"/>
+      <c r="AL18" s="63"/>
     </row>
     <row r="19" spans="1:42" ht="61.5" customHeight="1">
       <c r="A19" s="17" t="s">
@@ -2529,9 +2478,9 @@
         <f t="shared" ref="AI19" si="3">SUM(B19:AF19)</f>
         <v>5</v>
       </c>
-      <c r="AK19" s="69"/>
-      <c r="AL19" s="70"/>
-      <c r="AP19" s="67"/>
+      <c r="AK19" s="64"/>
+      <c r="AL19" s="63"/>
+      <c r="AP19" s="48"/>
     </row>
     <row r="20" spans="1:42" ht="61.5" customHeight="1">
       <c r="B20" s="25"/>
@@ -2566,11 +2515,11 @@
       <c r="AE20" s="25"/>
       <c r="AF20" s="25"/>
       <c r="AG20" s="5"/>
-      <c r="AK20" s="69"/>
-      <c r="AL20" s="70"/>
+      <c r="AK20" s="64"/>
+      <c r="AL20" s="63"/>
     </row>
     <row r="21" spans="1:42" ht="61.5" customHeight="1">
-      <c r="A21" s="64" t="s">
+      <c r="A21" s="54" t="s">
         <v>20</v>
       </c>
       <c r="B21" s="3">
@@ -2663,19 +2612,19 @@
       <c r="AE21" s="3">
         <v>30</v>
       </c>
-      <c r="AF21" s="48">
+      <c r="AF21" s="46">
         <v>31</v>
       </c>
       <c r="AG21" s="5"/>
-      <c r="AH21" s="60" t="s">
+      <c r="AH21" s="50" t="s">
         <v>20</v>
       </c>
-      <c r="AI21" s="61"/>
-      <c r="AK21" s="69"/>
-      <c r="AL21" s="70"/>
+      <c r="AI21" s="51"/>
+      <c r="AK21" s="64"/>
+      <c r="AL21" s="63"/>
     </row>
     <row r="22" spans="1:42" ht="61.5" customHeight="1">
-      <c r="A22" s="65"/>
+      <c r="A22" s="55"/>
       <c r="B22" s="10" t="s">
         <v>3</v>
       </c>
@@ -2766,14 +2715,14 @@
       <c r="AE22" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="AF22" s="42" t="s">
+      <c r="AF22" s="40" t="s">
         <v>5</v>
       </c>
       <c r="AG22" s="5"/>
-      <c r="AH22" s="62"/>
-      <c r="AI22" s="63"/>
-      <c r="AK22" s="69"/>
-      <c r="AL22" s="70"/>
+      <c r="AH22" s="52"/>
+      <c r="AI22" s="53"/>
+      <c r="AK22" s="64"/>
+      <c r="AL22" s="63"/>
     </row>
     <row r="23" spans="1:42" ht="61.5" customHeight="1">
       <c r="A23" s="12" t="s">
@@ -2837,7 +2786,7 @@
       </c>
       <c r="AD23" s="10"/>
       <c r="AE23" s="10"/>
-      <c r="AF23" s="42">
+      <c r="AF23" s="40">
         <v>9.25</v>
       </c>
       <c r="AG23" s="5"/>
@@ -2848,8 +2797,8 @@
         <f>SUM(B23:AF23)</f>
         <v>138.75</v>
       </c>
-      <c r="AK23" s="69"/>
-      <c r="AL23" s="70"/>
+      <c r="AK23" s="64"/>
+      <c r="AL23" s="63"/>
     </row>
     <row r="24" spans="1:42" ht="61.5" customHeight="1">
       <c r="A24" s="17" t="s">
@@ -2861,13 +2810,13 @@
       <c r="E24" s="19"/>
       <c r="F24" s="21"/>
       <c r="G24" s="18"/>
-      <c r="H24" s="46"/>
+      <c r="H24" s="44"/>
       <c r="I24" s="20"/>
       <c r="J24" s="20"/>
       <c r="K24" s="19"/>
       <c r="L24" s="19"/>
       <c r="M24" s="21"/>
-      <c r="N24" s="46"/>
+      <c r="N24" s="44"/>
       <c r="O24" s="19"/>
       <c r="P24" s="20"/>
       <c r="Q24" s="20"/>
@@ -2880,14 +2829,14 @@
       <c r="V24" s="19"/>
       <c r="W24" s="20"/>
       <c r="X24" s="20"/>
-      <c r="Y24" s="47"/>
+      <c r="Y24" s="45"/>
       <c r="Z24" s="19"/>
       <c r="AA24" s="21"/>
       <c r="AB24" s="19"/>
       <c r="AC24" s="19"/>
       <c r="AD24" s="20"/>
       <c r="AE24" s="20"/>
-      <c r="AF24" s="45"/>
+      <c r="AF24" s="43"/>
       <c r="AG24" s="5"/>
       <c r="AH24" s="23" t="s">
         <v>12</v>
@@ -2896,8 +2845,8 @@
         <f t="shared" ref="AI24" si="4">SUM(B24:AF24)</f>
         <v>1</v>
       </c>
-      <c r="AK24" s="69"/>
-      <c r="AL24" s="70"/>
+      <c r="AK24" s="64"/>
+      <c r="AL24" s="63"/>
     </row>
     <row r="25" spans="1:42" ht="61.5" customHeight="1">
       <c r="B25" s="25"/>
@@ -2932,11 +2881,11 @@
       <c r="AE25" s="25"/>
       <c r="AF25" s="25"/>
       <c r="AG25" s="5"/>
-      <c r="AK25" s="69"/>
-      <c r="AL25" s="70"/>
+      <c r="AK25" s="64"/>
+      <c r="AL25" s="63"/>
     </row>
     <row r="26" spans="1:42" ht="61.5" customHeight="1">
-      <c r="A26" s="64" t="s">
+      <c r="A26" s="54" t="s">
         <v>21</v>
       </c>
       <c r="B26" s="2">
@@ -3031,15 +2980,15 @@
       </c>
       <c r="AF26" s="25"/>
       <c r="AG26" s="5"/>
-      <c r="AH26" s="60" t="s">
+      <c r="AH26" s="50" t="s">
         <v>21</v>
       </c>
-      <c r="AI26" s="61"/>
-      <c r="AK26" s="69"/>
-      <c r="AL26" s="70"/>
+      <c r="AI26" s="51"/>
+      <c r="AK26" s="64"/>
+      <c r="AL26" s="63"/>
     </row>
     <row r="27" spans="1:42" ht="61.5" customHeight="1">
-      <c r="A27" s="65"/>
+      <c r="A27" s="55"/>
       <c r="B27" s="8" t="s">
         <v>6</v>
       </c>
@@ -3132,10 +3081,10 @@
       </c>
       <c r="AF27" s="25"/>
       <c r="AG27" s="5"/>
-      <c r="AH27" s="62"/>
-      <c r="AI27" s="63"/>
-      <c r="AK27" s="69"/>
-      <c r="AL27" s="70"/>
+      <c r="AH27" s="52"/>
+      <c r="AI27" s="53"/>
+      <c r="AK27" s="64"/>
+      <c r="AL27" s="63"/>
     </row>
     <row r="28" spans="1:42" ht="61.5" customHeight="1">
       <c r="A28" s="12" t="s">
@@ -3214,8 +3163,8 @@
         <f>SUM(B28:AF28)</f>
         <v>157.25</v>
       </c>
-      <c r="AK28" s="69"/>
-      <c r="AL28" s="70"/>
+      <c r="AK28" s="64"/>
+      <c r="AL28" s="63"/>
     </row>
     <row r="29" spans="1:42" ht="61.5" customHeight="1">
       <c r="A29" s="17" t="s">
@@ -3260,8 +3209,8 @@
         <f t="shared" ref="AI29" si="5">SUM(B29:AF29)</f>
         <v>0</v>
       </c>
-      <c r="AK29" s="69"/>
-      <c r="AL29" s="70"/>
+      <c r="AK29" s="64"/>
+      <c r="AL29" s="63"/>
     </row>
     <row r="30" spans="1:42" ht="61.5" customHeight="1">
       <c r="B30" s="25"/>
@@ -3296,11 +3245,11 @@
       <c r="AE30" s="25"/>
       <c r="AF30" s="25"/>
       <c r="AG30" s="5"/>
-      <c r="AK30" s="69"/>
-      <c r="AL30" s="70"/>
+      <c r="AK30" s="64"/>
+      <c r="AL30" s="63"/>
     </row>
     <row r="31" spans="1:42" ht="61.5" customHeight="1">
-      <c r="A31" s="64" t="s">
+      <c r="A31" s="54" t="s">
         <v>22</v>
       </c>
       <c r="B31" s="2">
@@ -3397,15 +3346,15 @@
         <v>31</v>
       </c>
       <c r="AG31" s="5"/>
-      <c r="AH31" s="60" t="s">
+      <c r="AH31" s="50" t="s">
         <v>22</v>
       </c>
-      <c r="AI31" s="61"/>
-      <c r="AK31" s="69"/>
-      <c r="AL31" s="70"/>
+      <c r="AI31" s="51"/>
+      <c r="AK31" s="64"/>
+      <c r="AL31" s="63"/>
     </row>
     <row r="32" spans="1:42" ht="61.5" customHeight="1">
-      <c r="A32" s="65"/>
+      <c r="A32" s="55"/>
       <c r="B32" s="8" t="s">
         <v>8</v>
       </c>
@@ -3500,10 +3449,10 @@
         <v>3</v>
       </c>
       <c r="AG32" s="5"/>
-      <c r="AH32" s="62"/>
-      <c r="AI32" s="63"/>
-      <c r="AK32" s="69"/>
-      <c r="AL32" s="70"/>
+      <c r="AH32" s="52"/>
+      <c r="AI32" s="53"/>
+      <c r="AK32" s="64"/>
+      <c r="AL32" s="63"/>
     </row>
     <row r="33" spans="1:38" ht="61.5" customHeight="1">
       <c r="A33" s="12" t="s">
@@ -3552,8 +3501,8 @@
         <f>SUM(B33:AF33)</f>
         <v>18.5</v>
       </c>
-      <c r="AK33" s="69"/>
-      <c r="AL33" s="70"/>
+      <c r="AK33" s="64"/>
+      <c r="AL33" s="63"/>
     </row>
     <row r="34" spans="1:38" ht="61.5" customHeight="1">
       <c r="A34" s="17" t="s">
@@ -3636,8 +3585,8 @@
         <f t="shared" ref="AI34" si="6">SUM(B34:AF34)</f>
         <v>19</v>
       </c>
-      <c r="AK34" s="69"/>
-      <c r="AL34" s="70"/>
+      <c r="AK34" s="64"/>
+      <c r="AL34" s="63"/>
     </row>
     <row r="35" spans="1:38" ht="61.5" customHeight="1">
       <c r="B35" s="25"/>
@@ -3672,11 +3621,11 @@
       <c r="AE35" s="25"/>
       <c r="AF35" s="25"/>
       <c r="AG35" s="5"/>
-      <c r="AK35" s="69"/>
-      <c r="AL35" s="70"/>
+      <c r="AK35" s="64"/>
+      <c r="AL35" s="63"/>
     </row>
     <row r="36" spans="1:38" ht="61.5" customHeight="1">
-      <c r="A36" s="64" t="s">
+      <c r="A36" s="54" t="s">
         <v>23</v>
       </c>
       <c r="B36" s="1">
@@ -3773,15 +3722,15 @@
         <v>31</v>
       </c>
       <c r="AG36" s="5"/>
-      <c r="AH36" s="60" t="s">
+      <c r="AH36" s="50" t="s">
         <v>23</v>
       </c>
-      <c r="AI36" s="61"/>
-      <c r="AK36" s="69"/>
-      <c r="AL36" s="70"/>
+      <c r="AI36" s="51"/>
+      <c r="AK36" s="64"/>
+      <c r="AL36" s="63"/>
     </row>
     <row r="37" spans="1:38" ht="61.5" customHeight="1">
-      <c r="A37" s="65"/>
+      <c r="A37" s="55"/>
       <c r="B37" s="7" t="s">
         <v>4</v>
       </c>
@@ -3876,10 +3825,10 @@
         <v>6</v>
       </c>
       <c r="AG37" s="5"/>
-      <c r="AH37" s="62"/>
-      <c r="AI37" s="63"/>
-      <c r="AK37" s="69"/>
-      <c r="AL37" s="70"/>
+      <c r="AH37" s="52"/>
+      <c r="AI37" s="53"/>
+      <c r="AK37" s="64"/>
+      <c r="AL37" s="63"/>
     </row>
     <row r="38" spans="1:38" ht="61.5" customHeight="1">
       <c r="A38" s="12" t="s">
@@ -3968,8 +3917,8 @@
         <f>SUM(B38:AF38)</f>
         <v>170.5</v>
       </c>
-      <c r="AK38" s="69"/>
-      <c r="AL38" s="70"/>
+      <c r="AK38" s="64"/>
+      <c r="AL38" s="63"/>
     </row>
     <row r="39" spans="1:38" ht="61.5" customHeight="1">
       <c r="A39" s="17" t="s">
@@ -4014,8 +3963,8 @@
         <f t="shared" ref="AI39" si="7">SUM(B39:AF39)</f>
         <v>0</v>
       </c>
-      <c r="AK39" s="69"/>
-      <c r="AL39" s="70"/>
+      <c r="AK39" s="64"/>
+      <c r="AL39" s="63"/>
     </row>
     <row r="40" spans="1:38" ht="61.5" customHeight="1">
       <c r="B40" s="25"/>
@@ -4050,11 +3999,11 @@
       <c r="AE40" s="25"/>
       <c r="AF40" s="25"/>
       <c r="AG40" s="5"/>
-      <c r="AK40" s="69"/>
-      <c r="AL40" s="70"/>
+      <c r="AK40" s="64"/>
+      <c r="AL40" s="63"/>
     </row>
     <row r="41" spans="1:38" ht="61.5" customHeight="1">
-      <c r="A41" s="64" t="s">
+      <c r="A41" s="54" t="s">
         <v>24</v>
       </c>
       <c r="B41" s="2">
@@ -4149,15 +4098,15 @@
       </c>
       <c r="AF41" s="34"/>
       <c r="AG41" s="5"/>
-      <c r="AH41" s="60" t="s">
+      <c r="AH41" s="50" t="s">
         <v>24</v>
       </c>
-      <c r="AI41" s="61"/>
-      <c r="AK41" s="69"/>
-      <c r="AL41" s="70"/>
+      <c r="AI41" s="51"/>
+      <c r="AK41" s="64"/>
+      <c r="AL41" s="63"/>
     </row>
     <row r="42" spans="1:38" ht="61.5" customHeight="1">
-      <c r="A42" s="65"/>
+      <c r="A42" s="55"/>
       <c r="B42" s="8" t="s">
         <v>7</v>
       </c>
@@ -4250,10 +4199,10 @@
       </c>
       <c r="AF42" s="34"/>
       <c r="AG42" s="5"/>
-      <c r="AH42" s="62"/>
-      <c r="AI42" s="63"/>
-      <c r="AK42" s="69"/>
-      <c r="AL42" s="70"/>
+      <c r="AH42" s="52"/>
+      <c r="AI42" s="53"/>
+      <c r="AK42" s="64"/>
+      <c r="AL42" s="63"/>
     </row>
     <row r="43" spans="1:38" ht="61.5" customHeight="1">
       <c r="A43" s="12" t="s">
@@ -4332,8 +4281,8 @@
         <f>SUM(B43:AF43)</f>
         <v>157.25</v>
       </c>
-      <c r="AK43" s="69"/>
-      <c r="AL43" s="70"/>
+      <c r="AK43" s="64"/>
+      <c r="AL43" s="63"/>
     </row>
     <row r="44" spans="1:38" ht="61.5" customHeight="1">
       <c r="A44" s="17" t="s">
@@ -4378,8 +4327,8 @@
         <f t="shared" ref="AI44" si="8">SUM(B44:AF44)</f>
         <v>0</v>
       </c>
-      <c r="AK44" s="69"/>
-      <c r="AL44" s="70"/>
+      <c r="AK44" s="64"/>
+      <c r="AL44" s="63"/>
     </row>
     <row r="45" spans="1:38" ht="61.5" customHeight="1">
       <c r="B45" s="25"/>
@@ -4414,11 +4363,11 @@
       <c r="AE45" s="25"/>
       <c r="AF45" s="25"/>
       <c r="AG45" s="5"/>
-      <c r="AK45" s="68"/>
-      <c r="AL45" s="68"/>
+      <c r="AK45" s="49"/>
+      <c r="AL45" s="49"/>
     </row>
     <row r="46" spans="1:38" ht="61.5" customHeight="1">
-      <c r="A46" s="64" t="s">
+      <c r="A46" s="54" t="s">
         <v>25</v>
       </c>
       <c r="B46" s="2">
@@ -4515,15 +4464,15 @@
         <v>31</v>
       </c>
       <c r="AG46" s="5"/>
-      <c r="AH46" s="60" t="s">
+      <c r="AH46" s="50" t="s">
         <v>25</v>
       </c>
-      <c r="AI46" s="61"/>
-      <c r="AK46" s="68"/>
-      <c r="AL46" s="68"/>
+      <c r="AI46" s="51"/>
+      <c r="AK46" s="49"/>
+      <c r="AL46" s="49"/>
     </row>
     <row r="47" spans="1:38" ht="61.5" customHeight="1">
-      <c r="A47" s="65"/>
+      <c r="A47" s="55"/>
       <c r="B47" s="8" t="s">
         <v>2</v>
       </c>
@@ -4618,10 +4567,10 @@
         <v>4</v>
       </c>
       <c r="AG47" s="5"/>
-      <c r="AH47" s="62"/>
-      <c r="AI47" s="63"/>
-      <c r="AK47" s="68"/>
-      <c r="AL47" s="68"/>
+      <c r="AH47" s="52"/>
+      <c r="AI47" s="53"/>
+      <c r="AK47" s="49"/>
+      <c r="AL47" s="49"/>
     </row>
     <row r="48" spans="1:38" ht="61.5" customHeight="1">
       <c r="A48" s="12" t="s">
@@ -4692,8 +4641,8 @@
         <f>SUM(B48:AF48)</f>
         <v>120.75</v>
       </c>
-      <c r="AK48" s="68"/>
-      <c r="AL48" s="68"/>
+      <c r="AK48" s="49"/>
+      <c r="AL48" s="49"/>
     </row>
     <row r="49" spans="1:39" ht="61.5" customHeight="1">
       <c r="A49" s="17" t="s">
@@ -4748,8 +4697,8 @@
         <f t="shared" ref="AI49" si="9">SUM(B49:AF49)</f>
         <v>5</v>
       </c>
-      <c r="AK49" s="68"/>
-      <c r="AL49" s="68"/>
+      <c r="AK49" s="49"/>
+      <c r="AL49" s="49"/>
     </row>
     <row r="50" spans="1:39" ht="61.5" customHeight="1">
       <c r="B50" s="25"/>
@@ -4786,7 +4735,7 @@
       <c r="AG50" s="5"/>
     </row>
     <row r="51" spans="1:39" ht="61.5" customHeight="1">
-      <c r="A51" s="64" t="s">
+      <c r="A51" s="54" t="s">
         <v>26</v>
       </c>
       <c r="B51" s="1">
@@ -4881,13 +4830,13 @@
       </c>
       <c r="AF51" s="34"/>
       <c r="AG51" s="5"/>
-      <c r="AH51" s="60" t="s">
+      <c r="AH51" s="50" t="s">
         <v>26</v>
       </c>
-      <c r="AI51" s="61"/>
+      <c r="AI51" s="51"/>
     </row>
     <row r="52" spans="1:39" ht="61.5" customHeight="1">
-      <c r="A52" s="65"/>
+      <c r="A52" s="55"/>
       <c r="B52" s="7" t="s">
         <v>5</v>
       </c>
@@ -4980,8 +4929,8 @@
       </c>
       <c r="AF52" s="34"/>
       <c r="AG52" s="5"/>
-      <c r="AH52" s="62"/>
-      <c r="AI52" s="63"/>
+      <c r="AH52" s="52"/>
+      <c r="AI52" s="53"/>
     </row>
     <row r="53" spans="1:39" ht="61.5" customHeight="1">
       <c r="A53" s="12" t="s">
@@ -5140,7 +5089,7 @@
       <c r="AG55" s="5"/>
     </row>
     <row r="56" spans="1:39" ht="61.5" customHeight="1">
-      <c r="A56" s="64" t="s">
+      <c r="A56" s="54" t="s">
         <v>27</v>
       </c>
       <c r="B56" s="2">
@@ -5237,18 +5186,18 @@
         <v>31</v>
       </c>
       <c r="AG56" s="5"/>
-      <c r="AH56" s="60" t="s">
+      <c r="AH56" s="50" t="s">
         <v>27</v>
       </c>
-      <c r="AI56" s="61"/>
-      <c r="AK56" s="49" t="s">
+      <c r="AI56" s="51"/>
+      <c r="AK56" s="65" t="s">
         <v>28</v>
       </c>
-      <c r="AL56" s="50"/>
+      <c r="AL56" s="66"/>
       <c r="AM56" s="34"/>
     </row>
     <row r="57" spans="1:39" ht="61.5" customHeight="1">
-      <c r="A57" s="65"/>
+      <c r="A57" s="55"/>
       <c r="B57" s="8" t="s">
         <v>7</v>
       </c>
@@ -5343,10 +5292,15 @@
         <v>2</v>
       </c>
       <c r="AG57" s="5"/>
-      <c r="AH57" s="62"/>
-      <c r="AI57" s="63"/>
-      <c r="AK57" s="51"/>
-      <c r="AL57" s="52"/>
+      <c r="AH57" s="52"/>
+      <c r="AI57" s="53"/>
+      <c r="AK57" s="12" t="s">
+        <v>29</v>
+      </c>
+      <c r="AL57" s="16">
+        <f>1607-AL58</f>
+        <v>12.25</v>
+      </c>
       <c r="AM57" s="34"/>
     </row>
     <row r="58" spans="1:39" ht="61.5" customHeight="1">
@@ -5422,10 +5376,10 @@
         <f>SUM(B58:AF58)</f>
         <v>131.25</v>
       </c>
-      <c r="AK58" s="37" t="s">
+      <c r="AK58" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="AL58" s="38">
+      <c r="AL58" s="16">
         <f>SUM(AI3,AI8,AI13,AI18,AI23,AI28,AI33,AI38,AI43,AI48,AI53,AI58)</f>
         <v>1594.75</v>
       </c>
@@ -5483,7 +5437,7 @@
         <f t="shared" ref="AI59" si="11">SUM(B59:AF59)</f>
         <v>5</v>
       </c>
-      <c r="AK59" s="23" t="s">
+      <c r="AK59" s="17" t="s">
         <v>12</v>
       </c>
       <c r="AL59" s="29">
@@ -5493,14 +5447,13 @@
     </row>
   </sheetData>
   <mergeCells count="31">
-    <mergeCell ref="AH11:AI12"/>
-    <mergeCell ref="AH6:AI7"/>
-    <mergeCell ref="AH1:AI2"/>
-    <mergeCell ref="AH41:AI42"/>
-    <mergeCell ref="AH36:AI37"/>
-    <mergeCell ref="AH31:AI32"/>
-    <mergeCell ref="AH26:AI27"/>
-    <mergeCell ref="AH21:AI22"/>
+    <mergeCell ref="AK2:AL2"/>
+    <mergeCell ref="AK3:AL3"/>
+    <mergeCell ref="AK4:AL4"/>
+    <mergeCell ref="AK5:AL6"/>
+    <mergeCell ref="AL16:AL44"/>
+    <mergeCell ref="AK16:AK44"/>
+    <mergeCell ref="AK56:AL56"/>
     <mergeCell ref="AH56:AI57"/>
     <mergeCell ref="AH51:AI52"/>
     <mergeCell ref="A56:A57"/>
@@ -5517,13 +5470,14 @@
     <mergeCell ref="A51:A52"/>
     <mergeCell ref="AH46:AI47"/>
     <mergeCell ref="AH16:AI17"/>
-    <mergeCell ref="AK56:AL57"/>
-    <mergeCell ref="AK2:AL2"/>
-    <mergeCell ref="AK3:AL3"/>
-    <mergeCell ref="AK4:AL4"/>
-    <mergeCell ref="AK5:AL6"/>
-    <mergeCell ref="AL16:AL44"/>
-    <mergeCell ref="AK16:AK44"/>
+    <mergeCell ref="AH11:AI12"/>
+    <mergeCell ref="AH6:AI7"/>
+    <mergeCell ref="AH1:AI2"/>
+    <mergeCell ref="AH41:AI42"/>
+    <mergeCell ref="AH36:AI37"/>
+    <mergeCell ref="AH31:AI32"/>
+    <mergeCell ref="AH26:AI27"/>
+    <mergeCell ref="AH21:AI22"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="8" scale="95" orientation="landscape"/>

</xml_diff>